<commit_message>
set up brigades  but not saving as int
</commit_message>
<xml_diff>
--- a/Austerlitz/Turns/306EJun1808.xlsx
+++ b/Austerlitz/Turns/306EJun1808.xlsx
@@ -1,20 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\Austerlitz\Austerlitz\Turns\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0D1BA62-39A6-4442-BFD1-AACBD6682CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="190" yWindow="490" windowWidth="18880" windowHeight="6740"/>
+    <workbookView xWindow="26460" yWindow="1260" windowWidth="18060" windowHeight="20070" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="94">
   <si>
     <t>A U S T E R L I T Z</t>
   </si>
@@ -228,11 +247,80 @@
   <si>
     <t>(23) Change State Relationships  (State/New Relationship)</t>
   </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>305</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Line Infantry</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>41</t>
+  </si>
+  <si>
+    <t>4085</t>
+  </si>
+  <si>
+    <t>65</t>
+  </si>
+  <si>
+    <t>61</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
+    <t>4086</t>
+  </si>
+  <si>
+    <t>1049</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>4087</t>
+  </si>
+  <si>
+    <t>4088</t>
+  </si>
+  <si>
+    <t>301</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Light Infantry</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="11">
     <font>
       <sz val="11"/>
@@ -465,7 +553,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="40">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -482,21 +570,18 @@
     <xf numFmtId="1" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="1" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="3" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="1" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="1" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="6" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="1" fontId="6" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -521,7 +606,7 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -533,6 +618,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="5" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="6" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="6" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -548,6 +636,14 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -748,50 +844,50 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L308"/>
-  <sheetFormatPr defaultColWidth="11.2109375" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="3.5703125" customWidth="1"/>
-    <col min="2" max="6" width="7.140625" customWidth="1"/>
-    <col min="7" max="7" width="8.42578125" customWidth="1"/>
-    <col min="8" max="9" width="7.140625" customWidth="1"/>
-    <col min="10" max="10" width="28.78515625" customWidth="1"/>
-    <col min="11" max="11" width="2.85546875" customWidth="1"/>
-    <col min="12" max="12" width="40.640625" customWidth="1"/>
+    <col min="1" max="1" width="3.59765625" customWidth="1"/>
+    <col min="2" max="6" width="7.09765625" customWidth="1"/>
+    <col min="7" max="7" width="8.3984375" customWidth="1"/>
+    <col min="8" max="9" width="7.09765625" customWidth="1"/>
+    <col min="10" max="10" width="28.796875" customWidth="1"/>
+    <col min="11" max="11" width="2.8984375" customWidth="1"/>
+    <col min="12" max="12" width="40.59765625" customWidth="1"/>
   </cols>
   <sheetData>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="1">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
       <c r="K1" s="1"/>
       <c r="L1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="2">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
     </row>
@@ -828,17 +924,17 @@
         <v>3</v>
       </c>
       <c r="B5" s="4"/>
-      <c r="C5" s="36" t="s">
+      <c r="C5" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="37"/>
+      <c r="D5" s="34"/>
       <c r="E5" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F5" s="4"/>
-      <c r="G5" s="38"/>
-      <c r="H5" s="39"/>
-      <c r="I5" s="37"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="36"/>
+      <c r="I5" s="34"/>
       <c r="J5" s="4"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
@@ -854,9 +950,9 @@
         <v>7</v>
       </c>
       <c r="F6" s="4"/>
-      <c r="G6" s="38"/>
-      <c r="H6" s="39"/>
-      <c r="I6" s="37"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="36"/>
+      <c r="I6" s="34"/>
       <c r="J6" s="4"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
@@ -870,9 +966,9 @@
         <v>8</v>
       </c>
       <c r="F7" s="4"/>
-      <c r="G7" s="38"/>
-      <c r="H7" s="39"/>
-      <c r="I7" s="37"/>
+      <c r="G7" s="35"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="34"/>
       <c r="J7" s="4"/>
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
@@ -955,13 +1051,37 @@
       <c r="A12" s="4">
         <v>1</v>
       </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
+      <c r="B12" s="37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C12" s="37" t="inlineStr">
+        <is>
+          <t>301</t>
+        </is>
+      </c>
+      <c r="D12" s="38" t="inlineStr">
+        <is>
+          <t>528000</t>
+        </is>
+      </c>
+      <c r="E12" s="37" t="inlineStr">
+        <is>
+          <t>4800</t>
+        </is>
+      </c>
+      <c r="F12" s="37" t="inlineStr">
+        <is>
+          <t>896</t>
+        </is>
+      </c>
       <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>800</t>
+        </is>
+      </c>
       <c r="I12" s="10"/>
       <c r="K12" s="5"/>
       <c r="L12" s="5" t="str">
@@ -1015,13 +1135,37 @@
       <c r="A13" s="4">
         <v>2</v>
       </c>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
+      <c r="B13" s="37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>305</t>
+        </is>
+      </c>
+      <c r="D13" s="37" t="inlineStr">
+        <is>
+          <t>800000</t>
+        </is>
+      </c>
+      <c r="E13" s="37" t="inlineStr">
+        <is>
+          <t>5600</t>
+        </is>
+      </c>
+      <c r="F13" s="37" t="inlineStr">
+        <is>
+          <t>1664</t>
+        </is>
+      </c>
       <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>1600</t>
+        </is>
+      </c>
       <c r="I13" s="10"/>
       <c r="K13" s="5"/>
       <c r="L13" s="5" t="str">
@@ -1069,7 +1213,7 @@
       <c r="A16" s="4">
         <v>5</v>
       </c>
-      <c r="B16" s="11"/>
+      <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
@@ -1204,7 +1348,7 @@
       <c r="L23" s="5"/>
     </row>
     <row spans="1:12" ht="5.25" customHeight="1" outlineLevel="0" r="24">
-      <c r="A24" s="13"/>
+      <c r="A24" s="11"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -1221,8 +1365,8 @@
       <c r="A25" s="4">
         <v>1</v>
       </c>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
@@ -1273,8 +1417,8 @@
       <c r="A26" s="4">
         <v>2</v>
       </c>
-      <c r="B26" s="15"/>
-      <c r="C26" s="14"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="12"/>
       <c r="D26" s="4"/>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
@@ -1291,8 +1435,8 @@
       <c r="A27" s="4">
         <v>3</v>
       </c>
-      <c r="B27" s="15"/>
-      <c r="C27" s="14"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="12"/>
       <c r="D27" s="4"/>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
@@ -1309,8 +1453,8 @@
       <c r="A28" s="4">
         <v>4</v>
       </c>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
       <c r="D28" s="4"/>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
@@ -1327,8 +1471,8 @@
       <c r="A29" s="4">
         <v>5</v>
       </c>
-      <c r="B29" s="15"/>
-      <c r="C29" s="15"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
@@ -1345,8 +1489,8 @@
       <c r="A30" s="4">
         <v>6</v>
       </c>
-      <c r="B30" s="16"/>
-      <c r="C30" s="15"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
@@ -1425,15 +1569,47 @@
       <c r="A34" s="4">
         <v>1</v>
       </c>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
-      <c r="F34" s="10"/>
-      <c r="G34" s="11"/>
-      <c r="H34" s="11"/>
-      <c r="I34" s="11"/>
-      <c r="J34" s="11"/>
+      <c r="B34" s="37" t="inlineStr">
+        <is>
+          <t>301</t>
+        </is>
+      </c>
+      <c r="C34" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D34" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E34" s="37" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="F34" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G34" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H34" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I34" s="10"/>
+      <c r="J34" s="37" t="inlineStr">
+        <is>
+          <t>Light Infantry</t>
+        </is>
+      </c>
       <c r="K34" s="5"/>
       <c r="L34" s="5" t="str">
         <f t="shared" ref="L34:L41" si="2">IF(AND(B34="",C34="",D34="",E34="",F34="",G34="",H34="",I34="",J34=""),"",
@@ -1453,26 +1629,62 @@
 IF(AND(I34&lt;&gt;"",OR(C34="",D34="",E34="",F34="",G34="",H34="")),"Battalion 7 requires all previous battalions",
 IF(J34="","Name is required",
 IF(LEN(J34)&gt;15,"Name must not exceed 15 characters","Valid")))))))))))</f>
-        <v/>
+        <v>Valid</v>
       </c>
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="35">
       <c r="A35" s="4">
         <v>2</v>
       </c>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
-      <c r="I35" s="10"/>
-      <c r="J35" s="10"/>
+      <c r="B35" s="37" t="inlineStr">
+        <is>
+          <t>305</t>
+        </is>
+      </c>
+      <c r="C35" s="37" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D35" s="37" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E35" s="37" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="F35" s="37" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G35" s="37" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="H35" s="37" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I35" s="37" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J35" s="37" t="inlineStr">
+        <is>
+          <t>Line Infantry</t>
+        </is>
+      </c>
       <c r="K35" s="5"/>
       <c r="L35" s="5" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Valid</v>
       </c>
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="36">
@@ -1541,10 +1753,10 @@
       <c r="D39" s="10"/>
       <c r="E39" s="10"/>
       <c r="F39" s="10"/>
-      <c r="G39" s="17"/>
+      <c r="G39" s="14"/>
       <c r="H39" s="10"/>
       <c r="I39" s="10"/>
-      <c r="J39" s="17"/>
+      <c r="J39" s="14"/>
       <c r="K39" s="5"/>
       <c r="L39" s="5" t="str">
         <f t="shared" si="2"/>
@@ -1620,7 +1832,7 @@
       <c r="L43" s="5"/>
     </row>
     <row spans="1:12" ht="5.25" customHeight="1" outlineLevel="0" r="44">
-      <c r="A44" s="13"/>
+      <c r="A44" s="11"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
@@ -1690,8 +1902,8 @@
       <c r="A47" s="4">
         <v>3</v>
       </c>
-      <c r="B47" s="17"/>
-      <c r="C47" s="17"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
       <c r="D47" s="4"/>
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
@@ -1709,8 +1921,8 @@
       <c r="A48" s="4">
         <v>4</v>
       </c>
-      <c r="B48" s="17"/>
-      <c r="C48" s="17"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="14"/>
       <c r="D48" s="4"/>
       <c r="E48" s="4"/>
       <c r="F48" s="4"/>
@@ -1793,7 +2005,7 @@
       <c r="L52" s="5"/>
     </row>
     <row spans="1:12" ht="14.25" customHeight="1" outlineLevel="0" r="53">
-      <c r="A53" s="13"/>
+      <c r="A53" s="11"/>
       <c r="B53" s="7"/>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
@@ -1810,7 +2022,7 @@
       <c r="A54" s="4">
         <v>1</v>
       </c>
-      <c r="B54" s="17"/>
+      <c r="B54" s="14"/>
       <c r="C54" s="10"/>
       <c r="D54" s="4"/>
       <c r="E54" s="4"/>
@@ -1847,7 +2059,7 @@
       <c r="A55" s="4">
         <v>2</v>
       </c>
-      <c r="B55" s="17"/>
+      <c r="B55" s="14"/>
       <c r="C55" s="10"/>
       <c r="D55" s="4"/>
       <c r="E55" s="4"/>
@@ -1866,8 +2078,8 @@
       <c r="A56" s="4">
         <v>3</v>
       </c>
-      <c r="B56" s="17"/>
-      <c r="C56" s="17"/>
+      <c r="B56" s="14"/>
+      <c r="C56" s="14"/>
       <c r="D56" s="4"/>
       <c r="E56" s="4"/>
       <c r="F56" s="4"/>
@@ -2083,7 +2295,7 @@
       <c r="L67" s="5"/>
     </row>
     <row spans="1:12" ht="5.25" customHeight="1" outlineLevel="0" r="68">
-      <c r="A68" s="13"/>
+      <c r="A68" s="11"/>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
@@ -2299,7 +2511,7 @@
       <c r="A79" s="4">
         <v>11</v>
       </c>
-      <c r="B79" s="17"/>
+      <c r="B79" s="14"/>
       <c r="C79" s="4"/>
       <c r="D79" s="4"/>
       <c r="E79" s="4"/>
@@ -2552,7 +2764,7 @@
       <c r="B91" s="10"/>
       <c r="C91" s="10"/>
       <c r="D91" s="10"/>
-      <c r="E91" s="17"/>
+      <c r="E91" s="14"/>
       <c r="F91" s="4"/>
       <c r="G91" s="4"/>
       <c r="H91" s="4"/>
@@ -2826,7 +3038,7 @@
       <c r="L104" s="5"/>
     </row>
     <row spans="1:12" ht="5.25" customHeight="1" outlineLevel="0" r="105">
-      <c r="A105" s="13"/>
+      <c r="A105" s="11"/>
       <c r="B105" s="4"/>
       <c r="C105" s="4"/>
       <c r="D105" s="4"/>
@@ -2872,7 +3084,7 @@
       <c r="A107" s="4">
         <v>2</v>
       </c>
-      <c r="B107" s="17"/>
+      <c r="B107" s="14"/>
       <c r="C107" s="4"/>
       <c r="D107" s="4"/>
       <c r="E107" s="4"/>
@@ -2994,7 +3206,7 @@
       <c r="L113" s="5"/>
     </row>
     <row spans="1:12" ht="5.25" customHeight="1" outlineLevel="0" r="114">
-      <c r="A114" s="13"/>
+      <c r="A114" s="11"/>
       <c r="B114" s="4"/>
       <c r="C114" s="4"/>
       <c r="D114" s="4"/>
@@ -3013,9 +3225,9 @@
       </c>
       <c r="B115" s="10"/>
       <c r="C115" s="10"/>
-      <c r="D115" s="18"/>
-      <c r="E115" s="19"/>
-      <c r="F115" s="20"/>
+      <c r="D115" s="15"/>
+      <c r="E115" s="16"/>
+      <c r="F115" s="17"/>
       <c r="G115" s="4"/>
       <c r="H115" s="4"/>
       <c r="I115" s="4"/>
@@ -3045,9 +3257,9 @@
       </c>
       <c r="B116" s="10"/>
       <c r="C116" s="10"/>
-      <c r="D116" s="18"/>
-      <c r="E116" s="19"/>
-      <c r="F116" s="20"/>
+      <c r="D116" s="15"/>
+      <c r="E116" s="16"/>
+      <c r="F116" s="17"/>
       <c r="G116" s="4"/>
       <c r="H116" s="4"/>
       <c r="I116" s="4"/>
@@ -3076,10 +3288,10 @@
         <v>3</v>
       </c>
       <c r="B117" s="10"/>
-      <c r="C117" s="17"/>
-      <c r="D117" s="18"/>
-      <c r="E117" s="19"/>
-      <c r="F117" s="20"/>
+      <c r="C117" s="14"/>
+      <c r="D117" s="15"/>
+      <c r="E117" s="16"/>
+      <c r="F117" s="17"/>
       <c r="G117" s="4"/>
       <c r="H117" s="4"/>
       <c r="I117" s="4"/>
@@ -3108,10 +3320,10 @@
         <v>4</v>
       </c>
       <c r="B118" s="10"/>
-      <c r="C118" s="17"/>
-      <c r="D118" s="18"/>
-      <c r="E118" s="19"/>
-      <c r="F118" s="20"/>
+      <c r="C118" s="14"/>
+      <c r="D118" s="15"/>
+      <c r="E118" s="16"/>
+      <c r="F118" s="17"/>
       <c r="G118" s="4"/>
       <c r="H118" s="4"/>
       <c r="I118" s="4"/>
@@ -3140,10 +3352,10 @@
         <v>5</v>
       </c>
       <c r="B119" s="10"/>
-      <c r="C119" s="17"/>
-      <c r="D119" s="21"/>
-      <c r="E119" s="19"/>
-      <c r="F119" s="20"/>
+      <c r="C119" s="14"/>
+      <c r="D119" s="18"/>
+      <c r="E119" s="16"/>
+      <c r="F119" s="17"/>
       <c r="G119" s="4"/>
       <c r="H119" s="4"/>
       <c r="I119" s="4"/>
@@ -3172,10 +3384,10 @@
         <v>6</v>
       </c>
       <c r="B120" s="10"/>
-      <c r="C120" s="17"/>
-      <c r="D120" s="21"/>
-      <c r="E120" s="19"/>
-      <c r="F120" s="20"/>
+      <c r="C120" s="14"/>
+      <c r="D120" s="18"/>
+      <c r="E120" s="16"/>
+      <c r="F120" s="17"/>
       <c r="G120" s="4"/>
       <c r="H120" s="4"/>
       <c r="I120" s="4"/>
@@ -3204,10 +3416,10 @@
         <v>7</v>
       </c>
       <c r="B121" s="10"/>
-      <c r="C121" s="17"/>
-      <c r="D121" s="21"/>
-      <c r="E121" s="19"/>
-      <c r="F121" s="20"/>
+      <c r="C121" s="14"/>
+      <c r="D121" s="18"/>
+      <c r="E121" s="16"/>
+      <c r="F121" s="17"/>
       <c r="G121" s="4"/>
       <c r="H121" s="4"/>
       <c r="I121" s="4"/>
@@ -3237,9 +3449,9 @@
       </c>
       <c r="B122" s="10"/>
       <c r="C122" s="10"/>
-      <c r="D122" s="18"/>
-      <c r="E122" s="19"/>
-      <c r="F122" s="20"/>
+      <c r="D122" s="15"/>
+      <c r="E122" s="16"/>
+      <c r="F122" s="17"/>
       <c r="G122" s="4"/>
       <c r="H122" s="4"/>
       <c r="I122" s="4"/>
@@ -3294,7 +3506,7 @@
       <c r="L124" s="5"/>
     </row>
     <row spans="1:12" ht="5.25" customHeight="1" outlineLevel="0" r="125">
-      <c r="A125" s="13"/>
+      <c r="A125" s="11"/>
       <c r="B125" s="4"/>
       <c r="C125" s="4"/>
       <c r="D125" s="4"/>
@@ -3333,7 +3545,7 @@
       <c r="A127" s="4">
         <v>2</v>
       </c>
-      <c r="B127" s="17"/>
+      <c r="B127" s="14"/>
       <c r="C127" s="4"/>
       <c r="D127" s="4"/>
       <c r="E127" s="4"/>
@@ -3352,7 +3564,7 @@
       <c r="A128" s="4">
         <v>3</v>
       </c>
-      <c r="B128" s="17"/>
+      <c r="B128" s="14"/>
       <c r="C128" s="4"/>
       <c r="D128" s="4"/>
       <c r="E128" s="4"/>
@@ -3417,7 +3629,7 @@
       <c r="L131" s="5"/>
     </row>
     <row spans="1:12" ht="5.25" customHeight="1" outlineLevel="0" r="132">
-      <c r="A132" s="13"/>
+      <c r="A132" s="11"/>
       <c r="B132" s="4"/>
       <c r="C132" s="4"/>
       <c r="D132" s="4"/>
@@ -3555,7 +3767,7 @@
         <v>4</v>
       </c>
       <c r="B136" s="10"/>
-      <c r="C136" s="17"/>
+      <c r="C136" s="14"/>
       <c r="D136" s="4"/>
       <c r="E136" s="4"/>
       <c r="F136" s="4"/>
@@ -3634,7 +3846,7 @@
       <c r="A138" s="4">
         <v>6</v>
       </c>
-      <c r="B138" s="17"/>
+      <c r="B138" s="14"/>
       <c r="C138" s="10"/>
       <c r="D138" s="4"/>
       <c r="E138" s="4"/>
@@ -3675,7 +3887,7 @@
         <v>7</v>
       </c>
       <c r="B139" s="10"/>
-      <c r="C139" s="17"/>
+      <c r="C139" s="14"/>
       <c r="D139" s="4"/>
       <c r="E139" s="4"/>
       <c r="F139" s="4"/>
@@ -3741,7 +3953,7 @@
       <c r="L141" s="5"/>
     </row>
     <row spans="1:12" ht="5.25" customHeight="1" outlineLevel="0" r="142">
-      <c r="A142" s="13"/>
+      <c r="A142" s="11"/>
       <c r="B142" s="4"/>
       <c r="C142" s="4"/>
       <c r="D142" s="4"/>
@@ -3758,17 +3970,17 @@
       <c r="A143" s="4">
         <v>1</v>
       </c>
-      <c r="B143" s="10" t="inlineStr">
+      <c r="B143" s="37" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="C143" s="10" t="inlineStr">
+      <c r="C143" s="37" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="D143" s="10" t="inlineStr">
+      <c r="D143" s="37" t="inlineStr">
         <is>
           <t>36</t>
         </is>
@@ -3811,17 +4023,17 @@
       <c r="A144" s="4">
         <v>2</v>
       </c>
-      <c r="B144" s="10" t="inlineStr">
+      <c r="B144" s="37" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="C144" s="10" t="inlineStr">
+      <c r="C144" s="37" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="D144" s="10" t="inlineStr">
+      <c r="D144" s="37" t="inlineStr">
         <is>
           <t>40</t>
         </is>
@@ -3864,17 +4076,17 @@
       <c r="A145" s="4">
         <v>3</v>
       </c>
-      <c r="B145" s="17" t="inlineStr">
+      <c r="B145" s="39" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="C145" s="10" t="inlineStr">
+      <c r="C145" s="37" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="D145" s="10" t="inlineStr">
+      <c r="D145" s="37" t="inlineStr">
         <is>
           <t>41</t>
         </is>
@@ -3917,9 +4129,9 @@
       <c r="A146" s="4">
         <v>4</v>
       </c>
-      <c r="B146" s="17"/>
+      <c r="B146" s="14"/>
       <c r="C146" s="10"/>
-      <c r="D146" s="17"/>
+      <c r="D146" s="14"/>
       <c r="E146" s="4"/>
       <c r="F146" s="4"/>
       <c r="G146" s="4"/>
@@ -4003,9 +4215,9 @@
       <c r="C148" s="10"/>
       <c r="D148" s="10"/>
       <c r="E148" s="4"/>
-      <c r="F148" s="22"/>
-      <c r="G148" s="22"/>
-      <c r="H148" s="22"/>
+      <c r="F148" s="19"/>
+      <c r="G148" s="19"/>
+      <c r="H148" s="19"/>
       <c r="I148" s="4"/>
       <c r="J148" s="4"/>
       <c r="K148" s="5"/>
@@ -4044,9 +4256,9 @@
       <c r="C149" s="10"/>
       <c r="D149" s="10"/>
       <c r="E149" s="4"/>
-      <c r="F149" s="22"/>
-      <c r="G149" s="22"/>
-      <c r="H149" s="22"/>
+      <c r="F149" s="19"/>
+      <c r="G149" s="19"/>
+      <c r="H149" s="19"/>
       <c r="I149" s="4"/>
       <c r="J149" s="4"/>
       <c r="K149" s="5"/>
@@ -4085,9 +4297,9 @@
       <c r="C150" s="10"/>
       <c r="D150" s="10"/>
       <c r="E150" s="4"/>
-      <c r="F150" s="22"/>
-      <c r="G150" s="22"/>
-      <c r="H150" s="22"/>
+      <c r="F150" s="19"/>
+      <c r="G150" s="19"/>
+      <c r="H150" s="19"/>
       <c r="I150" s="4"/>
       <c r="J150" s="4"/>
       <c r="K150" s="5"/>
@@ -4126,9 +4338,9 @@
       <c r="C151" s="10"/>
       <c r="D151" s="10"/>
       <c r="E151" s="4"/>
-      <c r="F151" s="22"/>
-      <c r="G151" s="22"/>
-      <c r="H151" s="22"/>
+      <c r="F151" s="19"/>
+      <c r="G151" s="19"/>
+      <c r="H151" s="19"/>
       <c r="I151" s="4"/>
       <c r="J151" s="4"/>
       <c r="K151" s="5"/>
@@ -4167,9 +4379,9 @@
       <c r="C152" s="10"/>
       <c r="D152" s="10"/>
       <c r="E152" s="4"/>
-      <c r="F152" s="22"/>
-      <c r="G152" s="22"/>
-      <c r="H152" s="22"/>
+      <c r="F152" s="19"/>
+      <c r="G152" s="19"/>
+      <c r="H152" s="19"/>
       <c r="I152" s="4"/>
       <c r="J152" s="4"/>
       <c r="K152" s="5"/>
@@ -4231,7 +4443,7 @@
       <c r="L154" s="5"/>
     </row>
     <row spans="1:12" ht="5.25" customHeight="1" outlineLevel="0" r="155">
-      <c r="A155" s="13"/>
+      <c r="A155" s="11"/>
       <c r="B155" s="4"/>
       <c r="C155" s="4"/>
       <c r="D155" s="4"/>
@@ -4306,12 +4518,12 @@
       <c r="A157" s="4">
         <v>2</v>
       </c>
-      <c r="B157" s="10" t="inlineStr">
+      <c r="B157" s="37" t="inlineStr">
         <is>
           <t>4085</t>
         </is>
       </c>
-      <c r="C157" s="10" t="inlineStr">
+      <c r="C157" s="37" t="inlineStr">
         <is>
           <t>65</t>
         </is>
@@ -4372,12 +4584,12 @@
       <c r="A158" s="4">
         <v>3</v>
       </c>
-      <c r="B158" s="10" t="inlineStr">
+      <c r="B158" s="37" t="inlineStr">
         <is>
           <t>61</t>
         </is>
       </c>
-      <c r="C158" s="10" t="inlineStr">
+      <c r="C158" s="37" t="inlineStr">
         <is>
           <t>64</t>
         </is>
@@ -4438,16 +4650,8 @@
       <c r="A159" s="4">
         <v>4</v>
       </c>
-      <c r="B159" s="10" t="inlineStr">
-        <is>
-          <t>4242</t>
-        </is>
-      </c>
-      <c r="C159" s="10" t="inlineStr">
-        <is>
-          <t>64</t>
-        </is>
-      </c>
+      <c r="B159" s="37"/>
+      <c r="C159" s="37"/>
       <c r="D159" s="4"/>
       <c r="E159" s="4"/>
       <c r="F159" s="4"/>
@@ -4504,12 +4708,12 @@
       <c r="A160" s="4">
         <v>5</v>
       </c>
-      <c r="B160" s="10" t="inlineStr">
+      <c r="B160" s="37" t="inlineStr">
         <is>
           <t>4086</t>
         </is>
       </c>
-      <c r="C160" s="10" t="inlineStr">
+      <c r="C160" s="37" t="inlineStr">
         <is>
           <t>65</t>
         </is>
@@ -4570,12 +4774,12 @@
       <c r="A161" s="4">
         <v>6</v>
       </c>
-      <c r="B161" s="10" t="inlineStr">
+      <c r="B161" s="37" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C161" s="10" t="inlineStr">
+      <c r="C161" s="37" t="inlineStr">
         <is>
           <t>64</t>
         </is>
@@ -4636,12 +4840,12 @@
       <c r="A162" s="4">
         <v>7</v>
       </c>
-      <c r="B162" s="10" t="inlineStr">
+      <c r="B162" s="37" t="inlineStr">
         <is>
           <t>1049</t>
         </is>
       </c>
-      <c r="C162" s="10" t="inlineStr">
+      <c r="C162" s="37" t="inlineStr">
         <is>
           <t>11</t>
         </is>
@@ -4763,8 +4967,8 @@
       <c r="B164" s="10"/>
       <c r="C164" s="10"/>
       <c r="D164" s="4"/>
-      <c r="E164" s="22"/>
-      <c r="F164" s="22"/>
+      <c r="E164" s="19"/>
+      <c r="F164" s="19"/>
       <c r="G164" s="4"/>
       <c r="H164" s="4"/>
       <c r="I164" s="4"/>
@@ -4821,8 +5025,8 @@
       <c r="B165" s="10"/>
       <c r="C165" s="10"/>
       <c r="D165" s="4"/>
-      <c r="E165" s="22"/>
-      <c r="F165" s="22"/>
+      <c r="E165" s="19"/>
+      <c r="F165" s="19"/>
       <c r="G165" s="4"/>
       <c r="H165" s="4"/>
       <c r="I165" s="4"/>
@@ -4876,11 +5080,11 @@
       <c r="A166" s="4">
         <v>11</v>
       </c>
-      <c r="B166" s="17"/>
+      <c r="B166" s="14"/>
       <c r="C166" s="10"/>
       <c r="D166" s="4"/>
-      <c r="E166" s="22"/>
-      <c r="F166" s="22"/>
+      <c r="E166" s="19"/>
+      <c r="F166" s="19"/>
       <c r="G166" s="4"/>
       <c r="H166" s="4"/>
       <c r="I166" s="4"/>
@@ -4935,10 +5139,10 @@
         <v>12</v>
       </c>
       <c r="B167" s="10"/>
-      <c r="C167" s="17"/>
+      <c r="C167" s="14"/>
       <c r="D167" s="4"/>
-      <c r="E167" s="22"/>
-      <c r="F167" s="22"/>
+      <c r="E167" s="19"/>
+      <c r="F167" s="19"/>
       <c r="G167" s="4"/>
       <c r="H167" s="4"/>
       <c r="I167" s="4"/>
@@ -4995,8 +5199,8 @@
       <c r="B168" s="10"/>
       <c r="C168" s="10"/>
       <c r="D168" s="4"/>
-      <c r="E168" s="22"/>
-      <c r="F168" s="22"/>
+      <c r="E168" s="19"/>
+      <c r="F168" s="19"/>
       <c r="G168" s="4"/>
       <c r="H168" s="4"/>
       <c r="I168" s="4"/>
@@ -5053,8 +5257,8 @@
       <c r="B169" s="10"/>
       <c r="C169" s="10"/>
       <c r="D169" s="4"/>
-      <c r="E169" s="22"/>
-      <c r="F169" s="22"/>
+      <c r="E169" s="19"/>
+      <c r="F169" s="19"/>
       <c r="G169" s="4"/>
       <c r="H169" s="4"/>
       <c r="I169" s="4"/>
@@ -5111,8 +5315,8 @@
       <c r="B170" s="10"/>
       <c r="C170" s="10"/>
       <c r="D170" s="4"/>
-      <c r="E170" s="22"/>
-      <c r="F170" s="22"/>
+      <c r="E170" s="19"/>
+      <c r="F170" s="19"/>
       <c r="G170" s="4"/>
       <c r="H170" s="4"/>
       <c r="I170" s="4"/>
@@ -5169,8 +5373,8 @@
       <c r="B171" s="10"/>
       <c r="C171" s="10"/>
       <c r="D171" s="4"/>
-      <c r="E171" s="22"/>
-      <c r="F171" s="22"/>
+      <c r="E171" s="19"/>
+      <c r="F171" s="19"/>
       <c r="G171" s="4"/>
       <c r="H171" s="4"/>
       <c r="I171" s="4"/>
@@ -5227,8 +5431,8 @@
       <c r="B172" s="10"/>
       <c r="C172" s="10"/>
       <c r="D172" s="4"/>
-      <c r="E172" s="22"/>
-      <c r="F172" s="22"/>
+      <c r="E172" s="19"/>
+      <c r="F172" s="19"/>
       <c r="G172" s="4"/>
       <c r="H172" s="4"/>
       <c r="I172" s="4"/>
@@ -5285,8 +5489,8 @@
       <c r="B173" s="10"/>
       <c r="C173" s="10"/>
       <c r="D173" s="4"/>
-      <c r="E173" s="22"/>
-      <c r="F173" s="22"/>
+      <c r="E173" s="19"/>
+      <c r="F173" s="19"/>
       <c r="G173" s="4"/>
       <c r="H173" s="4"/>
       <c r="I173" s="4"/>
@@ -5343,8 +5547,8 @@
       <c r="B174" s="10"/>
       <c r="C174" s="10"/>
       <c r="D174" s="4"/>
-      <c r="E174" s="22"/>
-      <c r="F174" s="22"/>
+      <c r="E174" s="19"/>
+      <c r="F174" s="19"/>
       <c r="G174" s="4"/>
       <c r="H174" s="4"/>
       <c r="I174" s="4"/>
@@ -5401,8 +5605,8 @@
       <c r="B175" s="10"/>
       <c r="C175" s="10"/>
       <c r="D175" s="4"/>
-      <c r="E175" s="22"/>
-      <c r="F175" s="22"/>
+      <c r="E175" s="19"/>
+      <c r="F175" s="19"/>
       <c r="G175" s="4"/>
       <c r="H175" s="4"/>
       <c r="I175" s="4"/>
@@ -5459,8 +5663,8 @@
       <c r="B176" s="10"/>
       <c r="C176" s="10"/>
       <c r="D176" s="4"/>
-      <c r="E176" s="22"/>
-      <c r="F176" s="22"/>
+      <c r="E176" s="19"/>
+      <c r="F176" s="19"/>
       <c r="G176" s="4"/>
       <c r="H176" s="4"/>
       <c r="I176" s="4"/>
@@ -5541,7 +5745,7 @@
       <c r="L178" s="5"/>
     </row>
     <row spans="1:12" ht="5.25" customHeight="1" outlineLevel="0" r="179">
-      <c r="A179" s="13"/>
+      <c r="A179" s="11"/>
       <c r="B179" s="4"/>
       <c r="C179" s="4"/>
       <c r="D179" s="4"/>
@@ -5630,7 +5834,7 @@
       <c r="A183" s="4">
         <v>4</v>
       </c>
-      <c r="B183" s="17"/>
+      <c r="B183" s="14"/>
       <c r="C183" s="10"/>
       <c r="D183" s="4"/>
       <c r="E183" s="4"/>
@@ -5734,20 +5938,20 @@
       <c r="A188" s="4">
         <v>1</v>
       </c>
-      <c r="B188" s="17"/>
-      <c r="C188" s="17" t="s">
+      <c r="B188" s="14"/>
+      <c r="C188" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D188" s="17" t="s">
+      <c r="D188" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="E188" s="17" t="s">
+      <c r="E188" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="F188" s="17" t="s">
+      <c r="F188" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="G188" s="17" t="s">
+      <c r="G188" s="14" t="s">
         <v>48</v>
       </c>
       <c r="H188" s="4"/>
@@ -5773,20 +5977,20 @@
       <c r="A189" s="4">
         <v>2</v>
       </c>
-      <c r="B189" s="17"/>
-      <c r="C189" s="17" t="s">
+      <c r="B189" s="14"/>
+      <c r="C189" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D189" s="17" t="s">
+      <c r="D189" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="E189" s="17" t="s">
+      <c r="E189" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="F189" s="17" t="s">
+      <c r="F189" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="G189" s="17" t="s">
+      <c r="G189" s="14" t="s">
         <v>48</v>
       </c>
       <c r="H189" s="4"/>
@@ -5813,19 +6017,19 @@
         <v>3</v>
       </c>
       <c r="B190" s="10"/>
-      <c r="C190" s="17" t="s">
+      <c r="C190" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D190" s="17" t="s">
+      <c r="D190" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="E190" s="17" t="s">
+      <c r="E190" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="F190" s="17" t="s">
+      <c r="F190" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="G190" s="17" t="s">
+      <c r="G190" s="14" t="s">
         <v>48</v>
       </c>
       <c r="H190" s="4"/>
@@ -6043,8 +6247,8 @@
       <c r="A196" s="4">
         <v>3</v>
       </c>
-      <c r="B196" s="17"/>
-      <c r="C196" s="17"/>
+      <c r="B196" s="14"/>
+      <c r="C196" s="14"/>
       <c r="D196" s="10"/>
       <c r="E196" s="10"/>
       <c r="F196" s="4"/>
@@ -6604,7 +6808,7 @@
         <v>11</v>
       </c>
       <c r="B204" s="10"/>
-      <c r="C204" s="17"/>
+      <c r="C204" s="14"/>
       <c r="D204" s="10"/>
       <c r="E204" s="10"/>
       <c r="F204" s="4"/>
@@ -7221,7 +7425,7 @@
       <c r="A215" s="4">
         <v>1</v>
       </c>
-      <c r="B215" s="17" t="inlineStr">
+      <c r="B215" s="39" t="inlineStr">
         <is>
           <t>4087</t>
         </is>
@@ -7289,7 +7493,7 @@
       <c r="A216" s="4">
         <v>2</v>
       </c>
-      <c r="B216" s="10" t="inlineStr">
+      <c r="B216" s="37" t="inlineStr">
         <is>
           <t>4088</t>
         </is>
@@ -7421,11 +7625,7 @@
       <c r="A218" s="4">
         <v>4</v>
       </c>
-      <c r="B218" s="10" t="inlineStr">
-        <is>
-          <t>4256</t>
-        </is>
-      </c>
+      <c r="B218" s="10"/>
       <c r="C218" s="10"/>
       <c r="D218" s="10"/>
       <c r="E218" s="10"/>
@@ -7489,7 +7689,7 @@
       <c r="A219" s="4">
         <v>5</v>
       </c>
-      <c r="B219" s="10" t="inlineStr">
+      <c r="B219" s="37" t="inlineStr">
         <is>
           <t>4085</t>
         </is>
@@ -7814,12 +8014,12 @@
         <v>10</v>
       </c>
       <c r="B224" s="10"/>
-      <c r="C224" s="17"/>
+      <c r="C224" s="14"/>
       <c r="D224" s="10"/>
-      <c r="E224" s="17"/>
-      <c r="F224" s="17"/>
-      <c r="G224" s="17"/>
-      <c r="H224" s="17"/>
+      <c r="E224" s="14"/>
+      <c r="F224" s="14"/>
+      <c r="G224" s="14"/>
+      <c r="H224" s="14"/>
       <c r="I224" s="4"/>
       <c r="J224" s="4"/>
       <c r="K224" s="5"/>
@@ -10521,9 +10721,9 @@
       <c r="A269" s="4">
         <v>1</v>
       </c>
-      <c r="B269" s="23"/>
-      <c r="C269" s="17"/>
-      <c r="D269" s="17"/>
+      <c r="B269" s="20"/>
+      <c r="C269" s="14"/>
+      <c r="D269" s="14"/>
       <c r="E269" s="10"/>
       <c r="F269" s="4"/>
       <c r="G269" s="4"/>
@@ -10592,7 +10792,7 @@
       <c r="A270" s="4">
         <v>2</v>
       </c>
-      <c r="B270" s="23"/>
+      <c r="B270" s="20"/>
       <c r="C270" s="10"/>
       <c r="D270" s="10"/>
       <c r="E270" s="10"/>
@@ -10663,7 +10863,7 @@
       <c r="A271" s="4">
         <v>3</v>
       </c>
-      <c r="B271" s="24"/>
+      <c r="B271" s="21"/>
       <c r="C271" s="10"/>
       <c r="D271" s="10"/>
       <c r="E271" s="10"/>
@@ -10734,7 +10934,7 @@
       <c r="A272" s="4">
         <v>4</v>
       </c>
-      <c r="B272" s="24"/>
+      <c r="B272" s="21"/>
       <c r="C272" s="10"/>
       <c r="D272" s="10"/>
       <c r="E272" s="10"/>
@@ -10805,7 +11005,7 @@
       <c r="A273" s="4">
         <v>5</v>
       </c>
-      <c r="B273" s="24"/>
+      <c r="B273" s="21"/>
       <c r="C273" s="10"/>
       <c r="D273" s="10"/>
       <c r="E273" s="10"/>
@@ -10876,7 +11076,7 @@
       <c r="A274" s="4">
         <v>6</v>
       </c>
-      <c r="B274" s="24"/>
+      <c r="B274" s="21"/>
       <c r="C274" s="10"/>
       <c r="D274" s="10"/>
       <c r="E274" s="10"/>
@@ -10947,7 +11147,7 @@
       <c r="A275" s="4">
         <v>7</v>
       </c>
-      <c r="B275" s="24"/>
+      <c r="B275" s="21"/>
       <c r="C275" s="10"/>
       <c r="D275" s="10"/>
       <c r="E275" s="10"/>
@@ -11018,7 +11218,7 @@
       <c r="A276" s="4">
         <v>8</v>
       </c>
-      <c r="B276" s="24"/>
+      <c r="B276" s="21"/>
       <c r="C276" s="10"/>
       <c r="D276" s="10"/>
       <c r="E276" s="10"/>
@@ -11089,7 +11289,7 @@
       <c r="A277" s="4">
         <v>9</v>
       </c>
-      <c r="B277" s="24"/>
+      <c r="B277" s="21"/>
       <c r="C277" s="10"/>
       <c r="D277" s="10"/>
       <c r="E277" s="10"/>
@@ -11160,7 +11360,7 @@
       <c r="A278" s="4">
         <v>10</v>
       </c>
-      <c r="B278" s="24"/>
+      <c r="B278" s="21"/>
       <c r="C278" s="10"/>
       <c r="D278" s="10"/>
       <c r="E278" s="10"/>
@@ -11231,7 +11431,7 @@
       <c r="A279" s="4">
         <v>11</v>
       </c>
-      <c r="B279" s="24"/>
+      <c r="B279" s="21"/>
       <c r="C279" s="10"/>
       <c r="D279" s="10"/>
       <c r="E279" s="10"/>
@@ -11302,7 +11502,7 @@
       <c r="A280" s="4">
         <v>12</v>
       </c>
-      <c r="B280" s="24"/>
+      <c r="B280" s="21"/>
       <c r="C280" s="10"/>
       <c r="D280" s="10"/>
       <c r="E280" s="10"/>
@@ -11373,7 +11573,7 @@
       <c r="A281" s="4">
         <v>13</v>
       </c>
-      <c r="B281" s="24"/>
+      <c r="B281" s="21"/>
       <c r="C281" s="10"/>
       <c r="D281" s="10"/>
       <c r="E281" s="10"/>
@@ -11444,7 +11644,7 @@
       <c r="A282" s="4">
         <v>14</v>
       </c>
-      <c r="B282" s="24"/>
+      <c r="B282" s="21"/>
       <c r="C282" s="10"/>
       <c r="D282" s="10"/>
       <c r="E282" s="10"/>
@@ -11515,7 +11715,7 @@
       <c r="A283" s="4">
         <v>15</v>
       </c>
-      <c r="B283" s="24"/>
+      <c r="B283" s="21"/>
       <c r="C283" s="10"/>
       <c r="D283" s="10"/>
       <c r="E283" s="10"/>
@@ -11586,7 +11786,7 @@
       <c r="A284" s="4">
         <v>16</v>
       </c>
-      <c r="B284" s="24"/>
+      <c r="B284" s="21"/>
       <c r="C284" s="10"/>
       <c r="D284" s="10"/>
       <c r="E284" s="10"/>
@@ -11705,10 +11905,10 @@
       <c r="A288" s="4">
         <v>1</v>
       </c>
-      <c r="B288" s="14" t="s">
+      <c r="B288" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C288" s="25"/>
+      <c r="C288" s="22"/>
       <c r="D288" s="4"/>
       <c r="E288" s="4"/>
       <c r="F288" s="4"/>
@@ -11762,10 +11962,10 @@
       <c r="A289" s="4">
         <v>2</v>
       </c>
-      <c r="B289" s="14" t="s">
+      <c r="B289" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C289" s="25"/>
+      <c r="C289" s="22"/>
       <c r="D289" s="4"/>
       <c r="E289" s="4"/>
       <c r="F289" s="4"/>
@@ -11819,10 +12019,10 @@
       <c r="A290" s="4">
         <v>3</v>
       </c>
-      <c r="B290" s="14" t="s">
+      <c r="B290" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C290" s="25"/>
+      <c r="C290" s="22"/>
       <c r="D290" s="4"/>
       <c r="E290" s="4"/>
       <c r="F290" s="4"/>
@@ -11876,10 +12076,10 @@
       <c r="A291" s="4">
         <v>4</v>
       </c>
-      <c r="B291" s="14" t="s">
+      <c r="B291" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C291" s="25"/>
+      <c r="C291" s="22"/>
       <c r="D291" s="4"/>
       <c r="E291" s="4"/>
       <c r="F291" s="4"/>
@@ -11933,10 +12133,10 @@
       <c r="A292" s="4">
         <v>5</v>
       </c>
-      <c r="B292" s="14" t="s">
+      <c r="B292" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C292" s="25"/>
+      <c r="C292" s="22"/>
       <c r="D292" s="4"/>
       <c r="E292" s="4"/>
       <c r="F292" s="4"/>
@@ -11990,10 +12190,10 @@
       <c r="A293" s="4">
         <v>6</v>
       </c>
-      <c r="B293" s="14" t="s">
+      <c r="B293" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C293" s="26"/>
+      <c r="C293" s="23"/>
       <c r="D293" s="4"/>
       <c r="E293" s="4"/>
       <c r="F293" s="4"/>
@@ -12095,13 +12295,13 @@
       <c r="A297" s="4">
         <v>1</v>
       </c>
-      <c r="B297" s="15"/>
-      <c r="C297" s="30"/>
-      <c r="D297" s="31"/>
-      <c r="E297" s="31"/>
-      <c r="F297" s="31"/>
-      <c r="G297" s="31"/>
-      <c r="H297" s="32"/>
+      <c r="B297" s="13"/>
+      <c r="C297" s="27"/>
+      <c r="D297" s="28"/>
+      <c r="E297" s="28"/>
+      <c r="F297" s="28"/>
+      <c r="G297" s="28"/>
+      <c r="H297" s="29"/>
       <c r="I297" s="4"/>
       <c r="J297" s="4"/>
       <c r="K297" s="5"/>
@@ -12127,13 +12327,13 @@
       <c r="A298" s="4">
         <v>2</v>
       </c>
-      <c r="B298" s="15"/>
-      <c r="C298" s="30"/>
-      <c r="D298" s="31"/>
-      <c r="E298" s="31"/>
-      <c r="F298" s="31"/>
-      <c r="G298" s="31"/>
-      <c r="H298" s="32"/>
+      <c r="B298" s="13"/>
+      <c r="C298" s="27"/>
+      <c r="D298" s="28"/>
+      <c r="E298" s="28"/>
+      <c r="F298" s="28"/>
+      <c r="G298" s="28"/>
+      <c r="H298" s="29"/>
       <c r="I298" s="4"/>
       <c r="J298" s="4"/>
       <c r="K298" s="5"/>
@@ -12159,13 +12359,13 @@
       <c r="A299" s="4">
         <v>3</v>
       </c>
-      <c r="B299" s="15"/>
-      <c r="C299" s="30"/>
-      <c r="D299" s="31"/>
-      <c r="E299" s="31"/>
-      <c r="F299" s="31"/>
-      <c r="G299" s="31"/>
-      <c r="H299" s="32"/>
+      <c r="B299" s="13"/>
+      <c r="C299" s="27"/>
+      <c r="D299" s="28"/>
+      <c r="E299" s="28"/>
+      <c r="F299" s="28"/>
+      <c r="G299" s="28"/>
+      <c r="H299" s="29"/>
       <c r="I299" s="4"/>
       <c r="J299" s="4"/>
       <c r="K299" s="5"/>
@@ -12191,13 +12391,13 @@
       <c r="A300" s="4">
         <v>4</v>
       </c>
-      <c r="B300" s="15"/>
-      <c r="C300" s="27"/>
-      <c r="D300" s="28"/>
-      <c r="E300" s="28"/>
-      <c r="F300" s="28"/>
-      <c r="G300" s="28"/>
-      <c r="H300" s="29"/>
+      <c r="B300" s="13"/>
+      <c r="C300" s="24"/>
+      <c r="D300" s="25"/>
+      <c r="E300" s="25"/>
+      <c r="F300" s="25"/>
+      <c r="G300" s="25"/>
+      <c r="H300" s="26"/>
       <c r="I300" s="4"/>
       <c r="J300" s="4"/>
       <c r="K300" s="5"/>
@@ -12250,7 +12450,7 @@
       <c r="L302" s="5"/>
     </row>
     <row spans="1:12" ht="5.25" customHeight="1" outlineLevel="0" r="303">
-      <c r="A303" s="13"/>
+      <c r="A303" s="11"/>
       <c r="B303" s="4"/>
       <c r="C303" s="4"/>
       <c r="D303" s="4"/>
@@ -12267,7 +12467,7 @@
       <c r="A304" s="4">
         <v>1</v>
       </c>
-      <c r="B304" s="17" t="s">
+      <c r="B304" s="14" t="s">
         <v>48</v>
       </c>
       <c r="C304" s="10"/>
@@ -12295,7 +12495,7 @@
       <c r="A305" s="4">
         <v>2</v>
       </c>
-      <c r="B305" s="17" t="s">
+      <c r="B305" s="14" t="s">
         <v>48</v>
       </c>
       <c r="C305" s="10"/>
@@ -12323,10 +12523,10 @@
       <c r="A306" s="4">
         <v>3</v>
       </c>
-      <c r="B306" s="17" t="s">
+      <c r="B306" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C306" s="17"/>
+      <c r="C306" s="14"/>
       <c r="D306" s="4"/>
       <c r="E306" s="4"/>
       <c r="F306" s="4"/>
@@ -12351,10 +12551,10 @@
       <c r="A307" s="4">
         <v>4</v>
       </c>
-      <c r="B307" s="17" t="s">
+      <c r="B307" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C307" s="17"/>
+      <c r="C307" s="14"/>
       <c r="D307" s="4"/>
       <c r="E307" s="4"/>
       <c r="F307" s="4"/>
@@ -12407,10 +12607,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C188:G190 B288:B293 B304:B307">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C188:G190 B288:B293 B304:B307" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"-,A,B,D,E,F,G,H,I,K,M,N,P,R,S,T,W"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C5">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C5" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Choose,A,B,D,E,F,G,H,I,K,M,N,P,R,S,T,W"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>